<commit_message>
Étale les temps estimés jusqu'à environ 23 minutes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SjSsUvYfWg3LPV8sLWWofN
</commit_message>
<xml_diff>
--- a/Classement_2.xlsx
+++ b/Classement_2.xlsx
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0.008587962962962962</v>
+        <v>0.00869212962962963</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0.008587962962962962</v>
+        <v>0.00880787037037037</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.008587962962962962</v>
+        <v>0.00880787037037037</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.008599537037037037</v>
+        <v>0.00880787037037037</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.008599537037037037</v>
+        <v>0.008877314814814815</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.008622685185185185</v>
+        <v>0.008958333333333334</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.008645833333333333</v>
+        <v>0.008958333333333334</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.008668981481481481</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="3" t="n"/>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>0.008680555555555556</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0.008680555555555556</v>
+        <v>0.009155092592592593</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>0.008726851851851852</v>
+        <v>0.009282407407407408</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>0.008738425925925926</v>
+        <v>0.009282407407407408</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>0.008738425925925926</v>
+        <v>0.009340277777777777</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>0.008796296296296297</v>
+        <v>0.009398148148148149</v>
       </c>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="3" t="n"/>
@@ -2239,7 +2239,7 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>0.008796296296296297</v>
+        <v>0.009398148148148149</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.008819444444444444</v>
+        <v>0.009456018518518518</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.008819444444444444</v>
+        <v>0.009525462962962963</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.008819444444444444</v>
+        <v>0.009606481481481481</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.008819444444444444</v>
+        <v>0.009606481481481481</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0.008831018518518519</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.008831018518518519</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>0.008831018518518519</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.008831018518518519</v>
+        <v>0.009768518518518518</v>
       </c>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="3" t="n"/>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0.008842592592592593</v>
+        <v>0.009814814814814814</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.008854166666666666</v>
+        <v>0.009895833333333333</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.008900462962962962</v>
+        <v>0.009895833333333333</v>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0.008923611111111111</v>
+        <v>0.009965277777777778</v>
       </c>
       <c r="G63" s="2" t="n"/>
       <c r="H63" s="3" t="n"/>
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0.008923611111111111</v>
+        <v>0.009965277777777778</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.008946759259259258</v>
+        <v>0.009965277777777778</v>
       </c>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="3" t="n"/>
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.008946759259259258</v>
+        <v>0.009965277777777778</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -2791,7 +2791,7 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0.008958333333333334</v>
+        <v>0.01005787037037037</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.008969907407407407</v>
+        <v>0.01005787037037037</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.008969907407407407</v>
+        <v>0.01018518518518519</v>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.008969907407407407</v>
+        <v>0.01018518518518519</v>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>0.008993055555555556</v>
+        <v>0.01028935185185185</v>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>0.009016203703703703</v>
+        <v>0.01028935185185185</v>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>0.009016203703703703</v>
+        <v>0.01028935185185185</v>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>0.009027777777777777</v>
+        <v>0.01028935185185185</v>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>0.009027777777777777</v>
+        <v>0.01038194444444444</v>
       </c>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="3" t="n"/>
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>0.009027777777777777</v>
+        <v>0.01047453703703704</v>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>0.009062499999999999</v>
+        <v>0.01047453703703704</v>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="F78" s="4" t="n">
-        <v>0.009085648148148148</v>
+        <v>0.01047453703703704</v>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.009085648148148148</v>
+        <v>0.01047453703703704</v>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
@@ -3251,7 +3251,7 @@
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>0.009131944444444444</v>
+        <v>0.0105787037037037</v>
       </c>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="3" t="inlineStr">
@@ -3283,7 +3283,7 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>0.009131944444444444</v>
+        <v>0.010625</v>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="F82" s="4" t="n">
-        <v>0.009131944444444444</v>
+        <v>0.01075231481481482</v>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>0.009143518518518518</v>
+        <v>0.01085648148148148</v>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
@@ -3391,7 +3391,7 @@
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>0.009143518518518518</v>
+        <v>0.0109837962962963</v>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>0.009143518518518518</v>
+        <v>0.0109837962962963</v>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>0.009143518518518518</v>
+        <v>0.0109837962962963</v>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>0.009155092592592593</v>
+        <v>0.01108796296296296</v>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
@@ -3535,7 +3535,7 @@
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>0.009155092592592593</v>
+        <v>0.01116898148148148</v>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>0.009189814814814816</v>
+        <v>0.01116898148148148</v>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>0.009212962962962963</v>
+        <v>0.01125</v>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>0.009247685185185185</v>
+        <v>0.01125</v>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
@@ -3679,7 +3679,7 @@
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>0.009247685185185185</v>
+        <v>0.0112962962962963</v>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="F93" s="4" t="n">
-        <v>0.009247685185185185</v>
+        <v>0.0112962962962963</v>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="F94" s="4" t="n">
-        <v>0.009270833333333334</v>
+        <v>0.01140046296296296</v>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="F95" s="4" t="n">
-        <v>0.009270833333333334</v>
+        <v>0.01140046296296296</v>
       </c>
       <c r="G95" s="2" t="n"/>
       <c r="H95" s="3" t="n"/>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="F96" s="4" t="n">
-        <v>0.009270833333333334</v>
+        <v>0.01144675925925926</v>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
@@ -3851,7 +3851,7 @@
         </is>
       </c>
       <c r="F97" s="4" t="n">
-        <v>0.009270833333333334</v>
+        <v>0.01149305555555555</v>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="F98" s="4" t="n">
-        <v>0.009293981481481481</v>
+        <v>0.0115625</v>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="F99" s="4" t="n">
-        <v>0.009293981481481481</v>
+        <v>0.01162037037037037</v>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="F100" s="4" t="n">
-        <v>0.009293981481481481</v>
+        <v>0.01162037037037037</v>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
@@ -3995,7 +3995,7 @@
         </is>
       </c>
       <c r="F101" s="4" t="n">
-        <v>0.00931712962962963</v>
+        <v>0.01162037037037037</v>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
@@ -4031,7 +4031,7 @@
         </is>
       </c>
       <c r="F102" s="4" t="n">
-        <v>0.00931712962962963</v>
+        <v>0.01168981481481481</v>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="F103" s="4" t="n">
-        <v>0.009340277777777777</v>
+        <v>0.01168981481481481</v>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
         </is>
       </c>
       <c r="F104" s="4" t="n">
-        <v>0.009340277777777777</v>
+        <v>0.01173611111111111</v>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>0.009340277777777777</v>
+        <v>0.01178240740740741</v>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="F106" s="4" t="n">
-        <v>0.009398148148148149</v>
+        <v>0.01178240740740741</v>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
@@ -4211,7 +4211,7 @@
         </is>
       </c>
       <c r="F107" s="4" t="n">
-        <v>0.009398148148148149</v>
+        <v>0.01184027777777778</v>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="F108" s="4" t="n">
-        <v>0.009432870370370371</v>
+        <v>0.01184027777777778</v>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
         </is>
       </c>
       <c r="F109" s="4" t="n">
-        <v>0.009467592592592593</v>
+        <v>0.01188657407407407</v>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="F110" s="4" t="n">
-        <v>0.009467592592592593</v>
+        <v>0.01196759259259259</v>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
@@ -4355,7 +4355,7 @@
         </is>
       </c>
       <c r="F111" s="4" t="n">
-        <v>0.009525462962962963</v>
+        <v>0.01196759259259259</v>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="F112" s="4" t="n">
-        <v>0.009525462962962963</v>
+        <v>0.01196759259259259</v>
       </c>
       <c r="G112" s="2" t="n"/>
       <c r="H112" s="3" t="n"/>
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="F113" s="4" t="n">
-        <v>0.009525462962962963</v>
+        <v>0.01201388888888889</v>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="F114" s="4" t="n">
-        <v>0.009537037037037037</v>
+        <v>0.01201388888888889</v>
       </c>
       <c r="G114" s="2" t="n"/>
       <c r="H114" s="3" t="n"/>
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="F115" s="4" t="n">
-        <v>0.009537037037037037</v>
+        <v>0.01201388888888889</v>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
@@ -4519,7 +4519,7 @@
         </is>
       </c>
       <c r="F116" s="4" t="n">
-        <v>0.009571759259259259</v>
+        <v>0.01212962962962963</v>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
@@ -4555,7 +4555,7 @@
         </is>
       </c>
       <c r="F117" s="4" t="n">
-        <v>0.009594907407407408</v>
+        <v>0.0122337962962963</v>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
@@ -4591,7 +4591,7 @@
         </is>
       </c>
       <c r="F118" s="4" t="n">
-        <v>0.009606481481481481</v>
+        <v>0.0122337962962963</v>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="F119" s="4" t="n">
-        <v>0.009641203703703704</v>
+        <v>0.01228009259259259</v>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
@@ -4663,7 +4663,7 @@
         </is>
       </c>
       <c r="F120" s="4" t="n">
-        <v>0.009652777777777777</v>
+        <v>0.01228009259259259</v>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
@@ -4699,7 +4699,7 @@
         </is>
       </c>
       <c r="F121" s="4" t="n">
-        <v>0.009652777777777777</v>
+        <v>0.01234953703703704</v>
       </c>
       <c r="G121" s="2" t="n"/>
       <c r="H121" s="3" t="n"/>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="F122" s="4" t="n">
-        <v>0.009699074074074074</v>
+        <v>0.01234953703703704</v>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
@@ -4763,7 +4763,7 @@
         </is>
       </c>
       <c r="F123" s="4" t="n">
-        <v>0.009722222222222222</v>
+        <v>0.01234953703703704</v>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
@@ -4799,7 +4799,7 @@
         </is>
       </c>
       <c r="F124" s="4" t="n">
-        <v>0.009722222222222222</v>
+        <v>0.01234953703703704</v>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
@@ -4835,7 +4835,7 @@
         </is>
       </c>
       <c r="F125" s="4" t="n">
-        <v>0.009768518518518518</v>
+        <v>0.01241898148148148</v>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="F126" s="4" t="n">
-        <v>0.009768518518518518</v>
+        <v>0.01241898148148148</v>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="F127" s="4" t="n">
-        <v>0.009768518518518518</v>
+        <v>0.01241898148148148</v>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="F128" s="4" t="n">
-        <v>0.009814814814814814</v>
+        <v>0.0125</v>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
@@ -4979,7 +4979,7 @@
         </is>
       </c>
       <c r="F129" s="4" t="n">
-        <v>0.009837962962962963</v>
+        <v>0.01255787037037037</v>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="F130" s="4" t="n">
-        <v>0.009837962962962963</v>
+        <v>0.01255787037037037</v>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
@@ -5051,7 +5051,7 @@
         </is>
       </c>
       <c r="F131" s="4" t="n">
-        <v>0.009884259259259259</v>
+        <v>0.01255787037037037</v>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="F132" s="4" t="n">
-        <v>0.009884259259259259</v>
+        <v>0.01255787037037037</v>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
         </is>
       </c>
       <c r="F133" s="4" t="n">
-        <v>0.009884259259259259</v>
+        <v>0.01267361111111111</v>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
@@ -5159,7 +5159,7 @@
         </is>
       </c>
       <c r="F134" s="4" t="n">
-        <v>0.009884259259259259</v>
+        <v>0.01280092592592593</v>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="F135" s="4" t="n">
-        <v>0.009895833333333333</v>
+        <v>0.01280092592592593</v>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="F136" s="4" t="n">
-        <v>0.009907407407407408</v>
+        <v>0.01288194444444444</v>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="F137" s="4" t="n">
-        <v>0.009930555555555555</v>
+        <v>0.01288194444444444</v>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
@@ -5303,7 +5303,7 @@
         </is>
       </c>
       <c r="F138" s="4" t="n">
-        <v>0.009930555555555555</v>
+        <v>0.01288194444444444</v>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
@@ -5339,7 +5339,7 @@
         </is>
       </c>
       <c r="F139" s="4" t="n">
-        <v>0.009942129629629629</v>
+        <v>0.01297453703703704</v>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
         </is>
       </c>
       <c r="F140" s="4" t="n">
-        <v>0.009965277777777778</v>
+        <v>0.01302083333333333</v>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
@@ -5411,7 +5411,7 @@
         </is>
       </c>
       <c r="F141" s="4" t="n">
-        <v>0.009965277777777778</v>
+        <v>0.01302083333333333</v>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
@@ -5447,7 +5447,7 @@
         </is>
       </c>
       <c r="F142" s="4" t="n">
-        <v>0.009988425925925927</v>
+        <v>0.0130787037037037</v>
       </c>
       <c r="G142" s="2" t="n"/>
       <c r="H142" s="3" t="n"/>
@@ -5475,7 +5475,7 @@
         </is>
       </c>
       <c r="F143" s="4" t="n">
-        <v>0.009988425925925927</v>
+        <v>0.01314814814814815</v>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="F144" s="4" t="n">
-        <v>0.009988425925925927</v>
+        <v>0.01314814814814815</v>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="F145" s="4" t="n">
-        <v>0.009988425925925927</v>
+        <v>0.01314814814814815</v>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
         </is>
       </c>
       <c r="F146" s="4" t="n">
-        <v>0.01002314814814815</v>
+        <v>0.01321759259259259</v>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="F147" s="4" t="n">
-        <v>0.01002314814814815</v>
+        <v>0.01321759259259259</v>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
@@ -5655,7 +5655,7 @@
         </is>
       </c>
       <c r="F148" s="4" t="n">
-        <v>0.01005787037037037</v>
+        <v>0.01321759259259259</v>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
@@ -5691,7 +5691,7 @@
         </is>
       </c>
       <c r="F149" s="4" t="n">
-        <v>0.01005787037037037</v>
+        <v>0.01333333333333333</v>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
@@ -5727,7 +5727,7 @@
         </is>
       </c>
       <c r="F150" s="4" t="n">
-        <v>0.01005787037037037</v>
+        <v>0.01333333333333333</v>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
@@ -5763,7 +5763,7 @@
         </is>
       </c>
       <c r="F151" s="4" t="n">
-        <v>0.01006944444444445</v>
+        <v>0.0133912037037037</v>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="F152" s="4" t="n">
-        <v>0.01006944444444445</v>
+        <v>0.0133912037037037</v>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
@@ -5835,7 +5835,7 @@
         </is>
       </c>
       <c r="F153" s="4" t="n">
-        <v>0.01006944444444445</v>
+        <v>0.0133912037037037</v>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
@@ -5867,7 +5867,7 @@
         </is>
       </c>
       <c r="F154" s="4" t="n">
-        <v>0.01006944444444445</v>
+        <v>0.0133912037037037</v>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
@@ -5903,7 +5903,7 @@
         </is>
       </c>
       <c r="F155" s="4" t="n">
-        <v>0.01010416666666667</v>
+        <v>0.01342592592592593</v>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
       <c r="F156" s="4" t="n">
-        <v>0.01010416666666667</v>
+        <v>0.01355324074074074</v>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
@@ -5975,7 +5975,7 @@
         </is>
       </c>
       <c r="F157" s="4" t="n">
-        <v>0.01010416666666667</v>
+        <v>0.01355324074074074</v>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
@@ -6011,7 +6011,7 @@
         </is>
       </c>
       <c r="F158" s="4" t="n">
-        <v>0.01010416666666667</v>
+        <v>0.01355324074074074</v>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
@@ -6047,7 +6047,7 @@
         </is>
       </c>
       <c r="F159" s="4" t="n">
-        <v>0.01013888888888889</v>
+        <v>0.01364583333333333</v>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="F160" s="4" t="n">
-        <v>0.01013888888888889</v>
+        <v>0.01364583333333333</v>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
@@ -6119,7 +6119,7 @@
         </is>
       </c>
       <c r="F161" s="4" t="n">
-        <v>0.01016203703703704</v>
+        <v>0.0137037037037037</v>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
       <c r="F162" s="4" t="n">
-        <v>0.01019675925925926</v>
+        <v>0.0137037037037037</v>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="F163" s="4" t="n">
-        <v>0.01020833333333333</v>
+        <v>0.0137962962962963</v>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="F164" s="4" t="n">
-        <v>0.01021990740740741</v>
+        <v>0.0137962962962963</v>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="E165" s="3" t="n"/>
       <c r="F165" s="4" t="n">
-        <v>0.01023148148148148</v>
+        <v>0.01384259259259259</v>
       </c>
       <c r="G165" s="2" t="n"/>
       <c r="H165" s="3" t="n"/>
@@ -6287,7 +6287,7 @@
         </is>
       </c>
       <c r="F166" s="4" t="n">
-        <v>0.01024305555555556</v>
+        <v>0.01384259259259259</v>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
         </is>
       </c>
       <c r="F167" s="4" t="n">
-        <v>0.0102662037037037</v>
+        <v>0.01384259259259259</v>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="F168" s="4" t="n">
-        <v>0.0103125</v>
+        <v>0.01393518518518519</v>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
@@ -6395,7 +6395,7 @@
         </is>
       </c>
       <c r="F169" s="4" t="n">
-        <v>0.0103125</v>
+        <v>0.01393518518518519</v>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
@@ -6431,7 +6431,7 @@
         </is>
       </c>
       <c r="F170" s="4" t="n">
-        <v>0.01032407407407407</v>
+        <v>0.01393518518518519</v>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
@@ -6467,7 +6467,7 @@
         </is>
       </c>
       <c r="F171" s="4" t="n">
-        <v>0.01034722222222222</v>
+        <v>0.01393518518518519</v>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
@@ -6503,7 +6503,7 @@
         </is>
       </c>
       <c r="F172" s="4" t="n">
-        <v>0.01034722222222222</v>
+        <v>0.0140625</v>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
@@ -6539,7 +6539,7 @@
         </is>
       </c>
       <c r="F173" s="4" t="n">
-        <v>0.0103587962962963</v>
+        <v>0.0140625</v>
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
@@ -6575,7 +6575,7 @@
         </is>
       </c>
       <c r="F174" s="4" t="n">
-        <v>0.0103587962962963</v>
+        <v>0.01417824074074074</v>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
         </is>
       </c>
       <c r="F175" s="4" t="n">
-        <v>0.0103587962962963</v>
+        <v>0.01417824074074074</v>
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
@@ -6647,7 +6647,7 @@
         </is>
       </c>
       <c r="F176" s="4" t="n">
-        <v>0.01041666666666667</v>
+        <v>0.01417824074074074</v>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
@@ -6683,7 +6683,7 @@
         </is>
       </c>
       <c r="F177" s="4" t="n">
-        <v>0.01041666666666667</v>
+        <v>0.01428240740740741</v>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
         </is>
       </c>
       <c r="F178" s="4" t="n">
-        <v>0.01043981481481481</v>
+        <v>0.01435185185185185</v>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
@@ -6755,7 +6755,7 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>0.01045138888888889</v>
+        <v>0.01435185185185185</v>
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
         </is>
       </c>
       <c r="F180" s="4" t="n">
-        <v>0.01046296296296296</v>
+        <v>0.01435185185185185</v>
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
@@ -6827,7 +6827,7 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>0.01046296296296296</v>
+        <v>0.0144212962962963</v>
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
@@ -6863,7 +6863,7 @@
         </is>
       </c>
       <c r="F182" s="4" t="n">
-        <v>0.01046296296296296</v>
+        <v>0.0144212962962963</v>
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
@@ -6899,7 +6899,7 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>0.01047453703703704</v>
+        <v>0.01447916666666667</v>
       </c>
       <c r="G183" s="2" t="n"/>
       <c r="H183" s="3" t="n"/>
@@ -6927,7 +6927,7 @@
         </is>
       </c>
       <c r="F184" s="4" t="n">
-        <v>0.01053240740740741</v>
+        <v>0.01447916666666667</v>
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
@@ -6963,7 +6963,7 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>0.01053240740740741</v>
+        <v>0.01447916666666667</v>
       </c>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="3" t="n"/>
@@ -6991,7 +6991,7 @@
         </is>
       </c>
       <c r="F186" s="4" t="n">
-        <v>0.01054398148148148</v>
+        <v>0.01447916666666667</v>
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
@@ -7027,7 +7027,7 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0.01054398148148148</v>
+        <v>0.01459490740740741</v>
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="F188" s="4" t="n">
-        <v>0.01055555555555556</v>
+        <v>0.01459490740740741</v>
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
@@ -7099,7 +7099,7 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>0.01055555555555556</v>
+        <v>0.01459490740740741</v>
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
@@ -7135,7 +7135,7 @@
         </is>
       </c>
       <c r="F190" s="4" t="n">
-        <v>0.01061342592592593</v>
+        <v>0.01467592592592593</v>
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
@@ -7171,7 +7171,7 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>0.01061342592592593</v>
+        <v>0.01479166666666667</v>
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
@@ -7207,7 +7207,7 @@
         </is>
       </c>
       <c r="F192" s="4" t="n">
-        <v>0.01061342592592593</v>
+        <v>0.01479166666666667</v>
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
@@ -7243,7 +7243,7 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>0.01061342592592593</v>
+        <v>0.01486111111111111</v>
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
@@ -7279,7 +7279,7 @@
         </is>
       </c>
       <c r="F194" s="4" t="n">
-        <v>0.01064814814814815</v>
+        <v>0.01486111111111111</v>
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
@@ -7315,7 +7315,7 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>0.0106712962962963</v>
+        <v>0.01486111111111111</v>
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
@@ -7351,7 +7351,7 @@
         </is>
       </c>
       <c r="F196" s="4" t="n">
-        <v>0.01070601851851852</v>
+        <v>0.01493055555555556</v>
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>0.01070601851851852</v>
+        <v>0.0150462962962963</v>
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
         </is>
       </c>
       <c r="F198" s="4" t="n">
-        <v>0.01074074074074074</v>
+        <v>0.0150462962962963</v>
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>0.01075231481481482</v>
+        <v>0.01517361111111111</v>
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="F200" s="4" t="n">
-        <v>0.01075231481481482</v>
+        <v>0.01528935185185185</v>
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
@@ -7531,7 +7531,7 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>0.01075231481481482</v>
+        <v>0.01540509259259259</v>
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
@@ -7567,7 +7567,7 @@
         </is>
       </c>
       <c r="F202" s="4" t="n">
-        <v>0.01081018518518518</v>
+        <v>0.01552083333333333</v>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>0.01081018518518518</v>
+        <v>0.01552083333333333</v>
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
@@ -7639,7 +7639,7 @@
         </is>
       </c>
       <c r="F204" s="4" t="n">
-        <v>0.01081018518518518</v>
+        <v>0.01552083333333333</v>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
@@ -7675,7 +7675,7 @@
         </is>
       </c>
       <c r="F205" s="4" t="n">
-        <v>0.01081018518518518</v>
+        <v>0.015625</v>
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         </is>
       </c>
       <c r="F206" s="4" t="n">
-        <v>0.01085648148148148</v>
+        <v>0.01568287037037037</v>
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="F207" s="4" t="n">
-        <v>0.01085648148148148</v>
+        <v>0.01577546296296296</v>
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
         </is>
       </c>
       <c r="F208" s="4" t="n">
-        <v>0.01085648148148148</v>
+        <v>0.01577546296296296</v>
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
@@ -7819,7 +7819,7 @@
         </is>
       </c>
       <c r="F209" s="4" t="n">
-        <v>0.0108912037037037</v>
+        <v>0.01584490740740741</v>
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
@@ -7855,7 +7855,7 @@
         </is>
       </c>
       <c r="F210" s="4" t="n">
-        <v>0.01091435185185185</v>
+        <v>0.01584490740740741</v>
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
@@ -7891,7 +7891,7 @@
         </is>
       </c>
       <c r="F211" s="4" t="n">
-        <v>0.01091435185185185</v>
+        <v>0.01584490740740741</v>
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="F212" s="4" t="n">
-        <v>0.01092592592592593</v>
+        <v>0.01584490740740741</v>
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
         </is>
       </c>
       <c r="F213" s="4" t="n">
-        <v>0.0109375</v>
+        <v>0.0158912037037037</v>
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         </is>
       </c>
       <c r="F214" s="4" t="n">
-        <v>0.01097222222222222</v>
+        <v>0.0159375</v>
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
@@ -8035,7 +8035,7 @@
         </is>
       </c>
       <c r="F215" s="4" t="n">
-        <v>0.01097222222222222</v>
+        <v>0.0159375</v>
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
@@ -8071,7 +8071,7 @@
         </is>
       </c>
       <c r="F216" s="4" t="n">
-        <v>0.01097222222222222</v>
+        <v>0.01600694444444445</v>
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         </is>
       </c>
       <c r="F217" s="4" t="n">
-        <v>0.01097222222222222</v>
+        <v>0.01600694444444445</v>
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         </is>
       </c>
       <c r="F218" s="4" t="n">
-        <v>0.01099537037037037</v>
+        <v>0.01607638888888889</v>
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
         </is>
       </c>
       <c r="F219" s="4" t="n">
-        <v>0.01099537037037037</v>
+        <v>0.01607638888888889</v>
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="F220" s="4" t="n">
-        <v>0.01099537037037037</v>
+        <v>0.01607638888888889</v>
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Complète le sexe et la catégorie des élèves manquants
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SjSsUvYfWg3LPV8sLWWofN
</commit_message>
<xml_diff>
--- a/Classement_2.xlsx
+++ b/Classement_2.xlsx
@@ -741,8 +741,16 @@
       <c r="F8" s="4" t="n">
         <v>0.006863425925925926</v>
       </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1057,8 +1065,16 @@
       <c r="F17" s="4" t="n">
         <v>0.007326388888888889</v>
       </c>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="3" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Sénior M</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1157,10 +1173,14 @@
       <c r="F20" s="4" t="n">
         <v>0.007627314814814815</v>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Minime 2 M</t>
+          <t>Sénior M</t>
         </is>
       </c>
     </row>
@@ -1509,10 +1529,14 @@
       <c r="F30" s="4" t="n">
         <v>0.008090277777777778</v>
       </c>
-      <c r="G30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Minime 2 M</t>
+          <t>Sénior M</t>
         </is>
       </c>
     </row>
@@ -1577,10 +1601,14 @@
       <c r="F32" s="4" t="n">
         <v>0.008287037037037037</v>
       </c>
-      <c r="G32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Minime 2 M</t>
+          <t>Sénior M</t>
         </is>
       </c>
     </row>
@@ -2005,8 +2033,16 @@
       <c r="F44" s="4" t="n">
         <v>0.009027777777777777</v>
       </c>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="3" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2213,8 +2249,16 @@
       <c r="F50" s="4" t="n">
         <v>0.009398148148148149</v>
       </c>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="3" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2529,8 +2573,16 @@
       <c r="F59" s="4" t="n">
         <v>0.009768518518518518</v>
       </c>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="3" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2665,8 +2717,16 @@
       <c r="F63" s="4" t="n">
         <v>0.009965277777777778</v>
       </c>
-      <c r="G63" s="2" t="n"/>
-      <c r="H63" s="3" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2729,8 +2789,16 @@
       <c r="F65" s="4" t="n">
         <v>0.009965277777777778</v>
       </c>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="3" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3081,8 +3149,16 @@
       <c r="F75" s="4" t="n">
         <v>0.01038194444444444</v>
       </c>
-      <c r="G75" s="2" t="n"/>
-      <c r="H75" s="3" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3253,10 +3329,14 @@
       <c r="F80" s="4" t="n">
         <v>0.0105787037037037</v>
       </c>
-      <c r="G80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>Cadet M</t>
+          <t>Sénior M</t>
         </is>
       </c>
     </row>
@@ -3789,8 +3869,16 @@
       <c r="F95" s="4" t="n">
         <v>0.01140046296296296</v>
       </c>
-      <c r="G95" s="2" t="n"/>
-      <c r="H95" s="3" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Sénior M</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -4393,8 +4481,16 @@
       <c r="F112" s="4" t="n">
         <v>0.01196759259259259</v>
       </c>
-      <c r="G112" s="2" t="n"/>
-      <c r="H112" s="3" t="n"/>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>Junior F</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -4457,8 +4553,16 @@
       <c r="F114" s="4" t="n">
         <v>0.01201388888888889</v>
       </c>
-      <c r="G114" s="2" t="n"/>
-      <c r="H114" s="3" t="n"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>Junior F</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -4701,8 +4805,16 @@
       <c r="F121" s="4" t="n">
         <v>0.01234953703703704</v>
       </c>
-      <c r="G121" s="2" t="n"/>
-      <c r="H121" s="3" t="n"/>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>Sénior M</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -5449,8 +5561,16 @@
       <c r="F142" s="4" t="n">
         <v>0.0130787037037037</v>
       </c>
-      <c r="G142" s="2" t="n"/>
-      <c r="H142" s="3" t="n"/>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -6261,7 +6381,11 @@
       <c r="F165" s="4" t="n">
         <v>0.01384259259259259</v>
       </c>
-      <c r="G165" s="2" t="n"/>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="H165" s="3" t="n"/>
     </row>
     <row r="166">
@@ -6901,8 +7025,16 @@
       <c r="F183" s="4" t="n">
         <v>0.01447916666666667</v>
       </c>
-      <c r="G183" s="2" t="n"/>
-      <c r="H183" s="3" t="n"/>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>Junior M</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -6965,8 +7097,16 @@
       <c r="F185" s="4" t="n">
         <v>0.01447916666666667</v>
       </c>
-      <c r="G185" s="2" t="n"/>
-      <c r="H185" s="3" t="n"/>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>Junior F</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">

</xml_diff>